<commit_message>
feat: add separate github action workflows for selenium, vulnerability, load, and appium testing, and configure dynamic load test reporting
</commit_message>
<xml_diff>
--- a/baseline_load_test_results.xlsx
+++ b/baseline_load_test_results.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Load Test Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Endpoint Details" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +53,14 @@
       <color rgb="00388E3C"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +85,12 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -149,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -164,7 +177,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -532,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -549,7 +571,6 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1"/>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -578,7 +599,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
@@ -591,7 +612,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>60 seconds</t>
+          <t>5.04 seconds</t>
         </is>
       </c>
       <c r="C7" s="5" t="n"/>
@@ -611,7 +632,6 @@
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -644,15 +664,15 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Total Duration</t>
+          <t>Total Duration (s)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>61.05</v>
+        <v>5.04</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>5s</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -668,7 +688,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>5293</v>
+        <v>331</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
@@ -688,7 +708,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>86.7</v>
+        <v>65.7</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
@@ -709,21 +729,20 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
@@ -760,7 +779,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>159.4</v>
+        <v>4</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
@@ -780,7 +799,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>1141.9</v>
+        <v>75.8</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
@@ -800,7 +819,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>3706.2</v>
+        <v>2165.2</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
@@ -813,7 +832,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
@@ -846,60 +864,20 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>HTTP 200 OK</t>
+          <t>HTTP 200</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>5293</v>
+        <v>331</v>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Successful responses</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>HTTP 500 Error</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Internal Server Errors</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Timeouts/Failures</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Network / Server connection errors</t>
         </is>
       </c>
     </row>
@@ -917,4 +895,201 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Endpoint-Level Performance Details (Load Test cases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Endpoint / Path</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Total Requests</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Passed Requests</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Failed Requests</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Min Latency (ms)</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Avg Latency (ms)</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Max Latency (ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>LOAD-EP-001</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>GET /health</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>2153.9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>LOAD-EP-002</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>GET /education/articles</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>83</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>83</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>2165.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>LOAD-EP-003</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>GET /education/faqs</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>2163.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>LOAD-EP-004</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>GET /diet/meal-templates</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>114.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>